<commit_message>
fix(office): preserve tables and extract DOCX charts
</commit_message>
<xml_diff>
--- a/tests/inputs/actors.xlsx
+++ b/tests/inputs/actors.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\serge\Storage\GoogleDrive\MyDrive\Я - ИТМО\Физика\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\serge\Storage\GitHub\hammerdown\tests\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B572ED1-99EB-4861-AC61-50115E978A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACE8C6A6-F5FC-46D1-9416-204216A98948}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B0B38B4A-8BD7-4786-AB65-6B3CC100DC9E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B0B38B4A-8BD7-4786-AB65-6B3CC100DC9E}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
+    <sheet name="Лист2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlchart.v1.0" hidden="1">Лист1!$D$1</definedName>
@@ -37,8 +38,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="242">
   <si>
     <t>№</t>
   </si>
@@ -758,6 +781,12 @@
   </si>
   <si>
     <t>Elena</t>
+  </si>
+  <si>
+    <t>Тестовые</t>
+  </si>
+  <si>
+    <t>формулы</t>
   </si>
 </sst>
 </file>
@@ -1796,7 +1825,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13DCA46F-8B16-4D6B-84FA-380C084F489D}">
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:O126"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4" bestFit="1" customWidth="1"/>
@@ -2044,7 +2073,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -2059,7 +2088,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -2074,7 +2103,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -2089,7 +2118,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -2104,7 +2133,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -2119,7 +2148,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -2134,7 +2163,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -2149,7 +2178,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -2164,7 +2193,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -2179,7 +2208,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -2194,7 +2223,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -2209,7 +2238,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="2">
         <v>27</v>
       </c>
@@ -2223,8 +2252,14 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="L28" t="s">
+        <v>240</v>
+      </c>
+      <c r="M28" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2238,8 +2273,16 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="L29" t="e">
+        <f>D19+B18</f>
+        <v>#VALUE!</v>
+      </c>
+      <c r="M29" t="str">
+        <f>B26</f>
+        <v>Di Sebastiani</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2253,8 +2296,22 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="L30" t="str">
+        <f>B21</f>
+        <v>Galano</v>
+      </c>
+      <c r="M30" t="str" cm="1">
+        <f t="array" ref="M30:O30">B1:D1</f>
+        <v>surname</v>
+      </c>
+      <c r="N30" t="str">
+        <v>name</v>
+      </c>
+      <c r="O30" t="str">
+        <v>len(name+surname)</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2269,7 +2326,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -3698,4 +3755,39 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26764F70-256C-4805-99C2-EE8BF556B96B}">
+  <dimension ref="C9:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="9" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C9" t="str" cm="1">
+        <f t="array" ref="C9:D11">Лист1!L28:M30</f>
+        <v>Тестовые</v>
+      </c>
+      <c r="D9" t="str">
+        <v>формулы</v>
+      </c>
+    </row>
+    <row r="10" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C10" t="e">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Di Sebastiani</v>
+      </c>
+    </row>
+    <row r="11" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C11" t="str">
+        <v>Galano</v>
+      </c>
+      <c r="D11" t="str">
+        <v>surname</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>